<commit_message>
feat: update performance analysis spreadsheet for Lambda document processing
</commit_message>
<xml_diff>
--- a/Lambda_Document_Processor_Performance_Analysis.xlsx
+++ b/Lambda_Document_Processor_Performance_Analysis.xlsx
@@ -1150,8 +1150,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1180,8 +1180,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1493,7 +1493,9 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1594,7 +1596,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19.7109375" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1818,7 +1830,11 @@
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2222,7 +2238,10 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2389,7 +2408,13 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.7109375" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="6" max="7" width="20.7109375" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -2547,7 +2572,12 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2680,7 +2710,8 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2814,7 +2845,11 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="6" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2947,7 +2982,12 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="26" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">

</xml_diff>

<commit_message>
feat: enable NaN and infinity error handling in performance analysis Excel report
</commit_message>
<xml_diff>
--- a/Lambda_Document_Processor_Performance_Analysis.xlsx
+++ b/Lambda_Document_Processor_Performance_Analysis.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="286">
   <si>
     <t>Metric</t>
   </si>
@@ -887,7 +887,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -899,14 +899,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -953,16 +945,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2925,90 +2914,170 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>145</v>
       </c>
+      <c r="D2" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E2" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F2" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>146</v>
       </c>
+      <c r="D3" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E3" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F3" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>151</v>
       </c>
+      <c r="E4" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F4" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B5" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>153</v>
       </c>
+      <c r="F5" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C6" t="s">
+      <c r="B6" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>152</v>
       </c>
+      <c r="E6" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F6" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C7" t="s">
+      <c r="B7" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F7" t="s">
+      <c r="D7" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E7" s="2" t="e">
+        <f>#NUM!</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>154</v>
       </c>
     </row>

</xml_diff>